<commit_message>
Shopee file follows the shared status doc: 5 single-piece SKUs
The status doc (21 Oct) says joints have not passed testing and 06 was never cut, so the Shopee
file now holds only the single-piece event SKUs (OC-01-01, OC-01-22, OC-03-26, OC-04-27, OC-05-28)
with SKU codes from the accounting sheet, and the text drops the no-sew and assembly claims.
24 and 29 stay out because they use 02. The prototype file is removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFe2Neq3JpzqWomS7eNDYn
</commit_message>
<xml_diff>
--- a/shopee-20261021/oct26-shopee-ready.xlsx
+++ b/shopee-20261021/oct26-shopee-ready.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4351" uniqueCount="4351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="4297">
   <si>
     <t>ภาพรวม</t>
   </si>
@@ -12819,16 +12819,16 @@
     <t>ps_new_size_chart_virtual_cat</t>
   </si>
   <si>
-    <t xml:space="preserve">ที่เก็บสายชาร์จหมี หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 ห้าหมี FIVE BEARS Love ของขวัญ</t>
+    <t xml:space="preserve">ที่เก็บสายชาร์จหมี หนังวัวแท้ งานแฮนด์เมด OCT. 26 ห้าหมี FIVE BEARS Love ของขวัญ</t>
   </si>
   <si>
     <t xml:space="preserve">สายชาร์จพันกันในกระเป๋าทุกวัน หมีตัวนี้ช่วยได้
 • คอลเลกชัน: ห้าหมี by OCT. 26 · Love
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: หัวหมี 01 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
+• วัสดุ: เศษหนังวัวแท้ หนา 1.0–1.2 มม. สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
+• ทำจาก: หัวหมี 01 × 1 ตัดด้วยบล็อกจากหนังแผ่นเดียว
 • ขนาด: 10.4 × 10.4 ซม.
 • เหมาะกับ: นักเรียน คนทำงาน
-วิธีประกอบ
+วิธีใช้
 1. พันสายชาร์จรอบหัวหมี
 2. เหน็บหัวปลั๊กเข้าร่องข้างแก้ม
 3. เหน็บอีกปลายเข้าร่องล่าง
@@ -12836,7 +12836,7 @@
 OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-01</t>
+    <t xml:space="preserve">OC-01-01</t>
   </si>
   <si>
     <t xml:space="preserve">59</t>
@@ -12845,7 +12845,7 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-01</t>
+    <t xml:space="preserve">OC-01-01</t>
   </si>
   <si>
     <t xml:space="preserve">https://oct26brand.com/assets/posters/01.png</t>
@@ -12857,168 +12857,16 @@
     <t xml:space="preserve">เปิด</t>
   </si>
   <si>
-    <t xml:space="preserve">ป้ายชื่อติดกระเป๋านักเรียน หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 ห้าหมี FIVE BEARS Love ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิดเทอมนี้ กระเป๋าลูกจะไม่หายไปกับของเพื่อน
-• คอลเลกชัน: ห้าหมี by OCT. 26 · Love
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: หัวหมี 01 × 1 + สายหัวใจ 250 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: หมี 10.4 ซม. สาย 25 ซม.
-• เหมาะกับ: ผู้ปกครอง
-วิธีประกอบ
-1. เขียนชื่อหลังหัวหมี
-2. ร้อยสายหัวใจผ่านร่องทั้งสอง
-3. คล้องหูกระเป๋าแล้วสอดปลายสายล็อก
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/03.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ห่วงผ้าเช็ดปากหมี หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 ห้าหมี FIVE BEARS Love ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">โต๊ะวันเกิดเด็กที่หมีนั่งเฝ้าทุกจาน
-• คอลเลกชัน: ห้าหมี by OCT. 26 · Love
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: หัวหมี 01 × 1 + สายหัวใจ 200 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: หมี 10.4 ซม.
-• เหมาะกับ: ร้านอาหาร งานวันเกิด
-วิธีประกอบ
-1. ร้อยสายสั้นผ่านร่องแก้มซ้าย
-2. อ้อมหลังแล้วร้อยร่องล่าง
-3. สอดผ้าเช็ดปากหรือช้อนส้อมเข้าห่วง
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">79</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/04.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ที่รองแก้วไส้ไม้ก๊อก หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">แก้วเย็นแค่ไหนโต๊ะก็ไม่เปียก
-• คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: วงกลม 05 × 2 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: 6.4 ซม.
-• เหมาะกับ: คาเฟ่ บาร์
-วิธีประกอบ
-1. วางไม้ก๊อกบนชิ้นล่าง
-2. ประกบชิ้นบน
-3. สอดปีกล็อกทั้งสี่ขอบ
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/15.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ของแขวนต้นคริสต์มาส หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ต้นคริสต์มาสปีนี้มีของแขวนหนังแท้
-• คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: กากบาทนุ่ม 06 × 6 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: 6 ซม.
-• เหมาะกับ: ช่วงปลายปี
-วิธีประกอบ
-1. เลือกหนังหลายสี
-2. ต่อเป็นลูกบาศก์
-3. ผูกริบบิ้นที่มุมบน
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">159</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/20.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ที่รองแก้วหมี หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 ห้าหมี FIVE BEARS Love ของขวัญ</t>
+    <t xml:space="preserve">ที่รองแก้วหมี หนังวัวแท้ งานแฮนด์เมด OCT. 26 ห้าหมี FIVE BEARS Love ของขวัญ</t>
   </si>
   <si>
     <t xml:space="preserve">แก้วนมตอนเช้ามีหมีรองอยู่
 • คอลเลกชัน: ห้าหมี by OCT. 26 · Love
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: หัวหมี 01 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
+• วัสดุ: เศษหนังวัวแท้ หนา 1.0–1.2 มม. สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
+• ทำจาก: หัวหมี 01 × 1 ตัดด้วยบล็อกจากหนังแผ่นเดียว
 • ขนาด: 10.4 ซม.
 • เหมาะกับ: ทุกบ้าน
-วิธีประกอบ
+วิธีใช้
 1. หยิบออกจากถุง
 2. วางแก้ว
 3. เสร็จ
@@ -13026,7 +12874,7 @@
 OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-22</t>
+    <t xml:space="preserve">OC-01-22</t>
   </si>
   <si>
     <t xml:space="preserve">59</t>
@@ -13035,7 +12883,7 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-22</t>
+    <t xml:space="preserve">OC-01-22</t>
   </si>
   <si>
     <t xml:space="preserve">https://oct26brand.com/assets/posters/22.png</t>
@@ -13047,54 +12895,16 @@
     <t xml:space="preserve">เปิด</t>
   </si>
   <si>
-    <t xml:space="preserve">ที่ห้อยกระเป๋าหมีหัวใจ หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 ห้าหมี FIVE BEARS Love ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">หมีห้อยกระเป๋าที่บอกว่าใครรักคุณอยู่
-• คอลเลกชัน: ห้าหมี by OCT. 26 · Love
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: หัวหมี 01 × 1 + สายหัวใจ 200 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: หมี 10.4 ซม.
-• เหมาะกับ: วัยรุ่น ของขวัญ
-วิธีประกอบ
-1. ร้อยห่วงโลหะที่ปลายสายหัวใจ
-2. สอดสายผ่านร่องแก้มและร่องล่าง
-3. คล้องห่วงกับกระเป๋า
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/23.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ป้ายห้อยของขวัญ หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
+    <t xml:space="preserve">ป้ายห้อยของขวัญ หนังวัวแท้ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
   </si>
   <si>
     <t xml:space="preserve">ป้ายชื่อที่ผู้รับเก็บไว้ห้อยกุญแจต่อได้
 • คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: กากบาทแคปซูล 03 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
+• วัสดุ: เศษหนังวัวแท้ หนา 1.0–1.2 มม. สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
+• ทำจาก: กากบาทแคปซูล 03 × 1 ตัดด้วยบล็อกจากหนังแผ่นเดียว
 • ขนาด: 9 ซม.
 • เหมาะกับ: ร้านของขวัญ
-วิธีประกอบ
+วิธีใช้
 1. เขียนชื่อผู้รับด้วยปากกาเพ้นท์
 2. ร้อยเชือกผ่านร่อง
 3. ผูกกับถุงของขวัญ
@@ -13102,7 +12912,7 @@
 OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-26</t>
+    <t xml:space="preserve">OC-03-26</t>
   </si>
   <si>
     <t xml:space="preserve">39</t>
@@ -13111,7 +12921,7 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-26</t>
+    <t xml:space="preserve">OC-03-26</t>
   </si>
   <si>
     <t xml:space="preserve">https://oct26brand.com/assets/posters/26.png</t>
@@ -13123,16 +12933,16 @@
     <t xml:space="preserve">เปิด</t>
   </si>
   <si>
-    <t xml:space="preserve">ที่รองแก้วสี่เหลี่ยม หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
+    <t xml:space="preserve">ที่รองแก้วสี่เหลี่ยม หนังวัวแท้ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
   </si>
   <si>
     <t xml:space="preserve">ที่รองแก้วทรงเหลี่ยมมน หนังแท้
 • คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: สี่เหลี่ยมมน 04 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
+• วัสดุ: เศษหนังวัวแท้ หนา 1.0–1.2 มม. สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
+• ทำจาก: สี่เหลี่ยมมน 04 × 1 ตัดด้วยบล็อกจากหนังแผ่นเดียว
 • ขนาด: 9 ซม.
 • เหมาะกับ: ทุกบ้าน
-วิธีประกอบ
+วิธีใช้
 1. หยิบออกจากถุง
 2. วางแก้ว
 3. เสร็จ
@@ -13140,7 +12950,7 @@
 OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-27</t>
+    <t xml:space="preserve">OC-04-27</t>
   </si>
   <si>
     <t xml:space="preserve">49</t>
@@ -13149,7 +12959,7 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-27</t>
+    <t xml:space="preserve">OC-04-27</t>
   </si>
   <si>
     <t xml:space="preserve">https://oct26brand.com/assets/posters/27.png</t>
@@ -13161,16 +12971,16 @@
     <t xml:space="preserve">เปิด</t>
   </si>
   <si>
-    <t xml:space="preserve">ที่รองแก้ววงกลม หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
+    <t xml:space="preserve">ที่รองแก้ววงกลม หนังวัวแท้ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
   </si>
   <si>
     <t xml:space="preserve">ที่รองแก้วทรงกลม หนังแท้
 • คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: วงกลม 05 × 1 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
+• วัสดุ: เศษหนังวัวแท้ หนา 1.0–1.2 มม. สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
+• ทำจาก: วงกลม 05 × 1 ตัดด้วยบล็อกจากหนังแผ่นเดียว
 • ขนาด: 9 ซม.
 • เหมาะกับ: ทุกบ้าน
-วิธีประกอบ
+วิธีใช้
 1. หยิบออกจากถุง
 2. วางแก้ว
 3. เสร็จ
@@ -13178,7 +12988,7 @@
 OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-28</t>
+    <t xml:space="preserve">OC-05-28</t>
   </si>
   <si>
     <t xml:space="preserve">49</t>
@@ -13187,51 +12997,13 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">OCT26-28</t>
+    <t xml:space="preserve">OC-05-28</t>
   </si>
   <si>
     <t xml:space="preserve">https://oct26brand.com/assets/posters/28.png</t>
   </si>
   <si>
     <t xml:space="preserve">0.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เปิด</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ชุดต่อเองกล่องลูกบาศก์ หนังแท้ ไม่ต้องเย็บ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ต่อเองได้ในห้านาที ไม่ต้องใช้กาว ไม่ต้องใช้เข็ม
-• คอลเลกชัน: OCT. 26 · SOI. 02
-• วัสดุ: เศษหนังวัวแท้ สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
-• ประกอบจาก: กากบาทนุ่ม 06 × 6 ต่อด้วยปีกและร่อง ไม่ใช้กาว ไม่เย็บ
-• ขนาด: 6 ซม. เมื่อต่อเสร็จ
-• เหมาะกับ: เด็ก ครอบครัว เวิร์กช็อป
-วิธีประกอบ
-1. เทชิ้นหนังหกชิ้นออกจากถุง
-2. ทำตามการ์ด ต่อ 4 ชิ้นเป็นวง
-3. ปิดก้นและฝา เสร็จในห้านาที
-การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
-OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCT26-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://oct26brand.com/assets/posters/30.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.2</t>
   </si>
   <si>
     <t xml:space="preserve">เปิด</t>
@@ -14309,7 +14081,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK17"/>
+  <dimension ref="A1:AK11"/>
   <cols>
     <col customWidth="true" max="37" min="37" style="8" width="20"/>
     <col customWidth="true" max="36" min="36" style="5" width="20"/>
@@ -15739,180 +15511,6 @@
         <v>4296</v>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="6" t="s">
-        <v>4297</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>4298</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>4299</v>
-      </c>
-      <c r="P12" s="6" t="s">
-        <v>4300</v>
-      </c>
-      <c r="Q12" s="5" t="s">
-        <v>4301</v>
-      </c>
-      <c r="R12" s="6" t="s">
-        <v>4302</v>
-      </c>
-      <c r="V12" s="6" t="s">
-        <v>4303</v>
-      </c>
-      <c r="AE12" s="6" t="s">
-        <v>4304</v>
-      </c>
-      <c r="AI12" s="6" t="s">
-        <v>4305</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="6" t="s">
-        <v>4306</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>4307</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>4308</v>
-      </c>
-      <c r="P13" s="6" t="s">
-        <v>4309</v>
-      </c>
-      <c r="Q13" s="5" t="s">
-        <v>4310</v>
-      </c>
-      <c r="R13" s="6" t="s">
-        <v>4311</v>
-      </c>
-      <c r="V13" s="6" t="s">
-        <v>4312</v>
-      </c>
-      <c r="AE13" s="6" t="s">
-        <v>4313</v>
-      </c>
-      <c r="AI13" s="6" t="s">
-        <v>4314</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="6" t="s">
-        <v>4315</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>4316</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>4317</v>
-      </c>
-      <c r="P14" s="6" t="s">
-        <v>4318</v>
-      </c>
-      <c r="Q14" s="5" t="s">
-        <v>4319</v>
-      </c>
-      <c r="R14" s="6" t="s">
-        <v>4320</v>
-      </c>
-      <c r="V14" s="6" t="s">
-        <v>4321</v>
-      </c>
-      <c r="AE14" s="6" t="s">
-        <v>4322</v>
-      </c>
-      <c r="AI14" s="6" t="s">
-        <v>4323</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="6" t="s">
-        <v>4324</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>4325</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>4326</v>
-      </c>
-      <c r="P15" s="6" t="s">
-        <v>4327</v>
-      </c>
-      <c r="Q15" s="5" t="s">
-        <v>4328</v>
-      </c>
-      <c r="R15" s="6" t="s">
-        <v>4329</v>
-      </c>
-      <c r="V15" s="6" t="s">
-        <v>4330</v>
-      </c>
-      <c r="AE15" s="6" t="s">
-        <v>4331</v>
-      </c>
-      <c r="AI15" s="6" t="s">
-        <v>4332</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="6" t="s">
-        <v>4333</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>4334</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>4335</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>4336</v>
-      </c>
-      <c r="Q16" s="5" t="s">
-        <v>4337</v>
-      </c>
-      <c r="R16" s="6" t="s">
-        <v>4338</v>
-      </c>
-      <c r="V16" s="6" t="s">
-        <v>4339</v>
-      </c>
-      <c r="AE16" s="6" t="s">
-        <v>4340</v>
-      </c>
-      <c r="AI16" s="6" t="s">
-        <v>4341</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="6" t="s">
-        <v>4342</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>4343</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>4344</v>
-      </c>
-      <c r="P17" s="6" t="s">
-        <v>4345</v>
-      </c>
-      <c r="Q17" s="5" t="s">
-        <v>4346</v>
-      </c>
-      <c r="R17" s="6" t="s">
-        <v>4347</v>
-      </c>
-      <c r="V17" s="6" t="s">
-        <v>4348</v>
-      </c>
-      <c r="AE17" s="6" t="s">
-        <v>4349</v>
-      </c>
-      <c r="AI17" s="6" t="s">
-        <v>4350</v>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection sheet="true" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Shopee: add OC-02-24 and OC-MX-29 as the owner decided
The shop is open with the first five SKUs, so oct26-shopee-add-24-29.xlsx carries only the two 02
products; oct26-shopee-ready.xlsx now holds all seven event SKUs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFe2Neq3JpzqWomS7eNDYn
</commit_message>
<xml_diff>
--- a/shopee-20261021/oct26-shopee-ready.xlsx
+++ b/shopee-20261021/oct26-shopee-ready.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="4297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4315" uniqueCount="4315">
   <si>
     <t>ภาพรวม</t>
   </si>
@@ -12895,6 +12895,44 @@
     <t xml:space="preserve">เปิด</t>
   </si>
   <si>
+    <t xml:space="preserve">ที่รองแก้วกังหัน หนังวัวแท้ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ที่รองแก้วลายกังหัน หนังแท้ทั้งแผ่น
+• คอลเลกชัน: OCT. 26 · SOI. 02
+• วัสดุ: เศษหนังวัวแท้ หนา 1.0–1.2 มม. สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
+• ทำจาก: กังหัน 02 × 1 ตัดด้วยบล็อกจากหนังแผ่นเดียว
+• ขนาด: 9 ซม.
+• เหมาะกับ: ทุกบ้าน
+วิธีใช้
+1. หยิบออกจากถุง
+2. วางแก้ว
+3. เสร็จ
+การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
+OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OC-02-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OC-02-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://oct26brand.com/assets/posters/24.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เปิด</t>
+  </si>
+  <si>
     <t xml:space="preserve">ป้ายห้อยของขวัญ หนังวัวแท้ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
   </si>
   <si>
@@ -13004,6 +13042,44 @@
   </si>
   <si>
     <t xml:space="preserve">0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เปิด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ชุดที่รองแก้ว 4 ลาย หนังวัวแท้ งานแฮนด์เมด OCT. 26 SOI. 02 ของขวัญ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สี่แก้ว สี่ลาย ไม่ต้องจำว่าแก้วไหนของใคร
+• คอลเลกชัน: OCT. 26 · SOI. 02
+• วัสดุ: เศษหนังวัวแท้ หนา 1.0–1.2 มม. สีและลายแต่ละชิ้นต่างกันเล็กน้อย ทุกชิ้นมีชิ้นเดียว
+• ทำจาก: หัวหมี 01 × 1 + กังหัน 02 × 1 + สี่เหลี่ยมมน 04 × 1 + วงกลม 05 × 1 แต่ละชิ้นตัดด้วยบล็อกจากหนังแผ่นเดียว
+• ขนาด: 9–10.4 ซม.
+• เหมาะกับ: ของขวัญขึ้นบ้านใหม่
+วิธีใช้
+1. เลือกสี่ลายที่ชอบ
+2. มัดรวมด้วยเชือกปอ
+3. ใส่ถุงผ้า
+การดูแล: เช็ดด้วยผ้าแห้ง เลี่ยงน้ำและแดดจัด
+OCT. 26 · our crafted things. ทำและแพ็คกันเองทั้งบ้าน พ่อ แม่ และลูกสามคน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OC-MX-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OC-MX-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://oct26brand.com/assets/posters/29.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2</t>
   </si>
   <si>
     <t xml:space="preserve">เปิด</t>
@@ -14081,7 +14157,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK11"/>
+  <dimension ref="A1:AK13"/>
   <cols>
     <col customWidth="true" max="37" min="37" style="8" width="20"/>
     <col customWidth="true" max="36" min="36" style="5" width="20"/>
@@ -15511,6 +15587,64 @@
         <v>4296</v>
       </c>
     </row>
+    <row r="12">
+      <c r="B12" s="6" t="s">
+        <v>4297</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>4298</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>4299</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>4300</v>
+      </c>
+      <c r="Q12" s="5" t="s">
+        <v>4301</v>
+      </c>
+      <c r="R12" s="6" t="s">
+        <v>4302</v>
+      </c>
+      <c r="V12" s="6" t="s">
+        <v>4303</v>
+      </c>
+      <c r="AE12" s="6" t="s">
+        <v>4304</v>
+      </c>
+      <c r="AI12" s="6" t="s">
+        <v>4305</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="6" t="s">
+        <v>4306</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>4307</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>4308</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>4309</v>
+      </c>
+      <c r="Q13" s="5" t="s">
+        <v>4310</v>
+      </c>
+      <c r="R13" s="6" t="s">
+        <v>4311</v>
+      </c>
+      <c r="V13" s="6" t="s">
+        <v>4312</v>
+      </c>
+      <c r="AE13" s="6" t="s">
+        <v>4313</v>
+      </c>
+      <c r="AI13" s="6" t="s">
+        <v>4314</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection sheet="true" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
   <dataValidations count="2">

</xml_diff>